<commit_message>
docs(knowledge): extend Bungalov 4KK knowledge from DSE web
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
+++ b/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
@@ -1408,7 +1408,21 @@
           <t>Jaká je užitná plocha domu?</t>
         </is>
       </c>
-      <c r="F65" s="12" t="n"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Užitná plocha domu je uvedena jako 129 m².</t>
+        </is>
+      </c>
+      <c r="F65" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="13">
       <c r="A66" s="8" t="n"/>
@@ -1423,7 +1437,21 @@
           <t>Jaká je zastavěná plocha domu?</t>
         </is>
       </c>
-      <c r="F66" s="12" t="n"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Zastavěná plocha domu je 119 m².</t>
+        </is>
+      </c>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="13">
       <c r="A67" s="8" t="n"/>
@@ -1498,7 +1526,26 @@
           <t>Jaká je celková velikost tohoto domu?</t>
         </is>
       </c>
-      <c r="F71" s="12" t="n"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Web uvádí u domu údaj 113 m², ale bez jednoznačného označení typu plochy.</t>
+        </is>
+      </c>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Zastavěná plocha 119 m² / Užitná plocha 129 m²</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="13">
       <c r="A72" s="8" t="n"/>
@@ -3199,7 +3246,21 @@
           <t>Jak se dům napojuje na elektřinu, vodu a kanalizaci?</t>
         </is>
       </c>
-      <c r="F200" s="12" t="n"/>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Referenční realizace má dálkový vodovod, elektřinu 230/400 V a biologickou čističku odpadních vod.</t>
+        </is>
+      </c>
+      <c r="F200" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="15.75" customHeight="1" s="13">
       <c r="C201" s="10" t="inlineStr">
@@ -3212,7 +3273,21 @@
           <t>Co když na pozemku není kanalizace?</t>
         </is>
       </c>
-      <c r="F201" s="12" t="n"/>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Referenční realizace používá biologickou čističku odpadních vod.</t>
+        </is>
+      </c>
+      <c r="F201" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="202" ht="15.75" customHeight="1" s="13">
       <c r="C202" s="10" t="inlineStr">
@@ -3316,7 +3391,21 @@
           <t>Jak se řeší dešťová voda ze střechy?</t>
         </is>
       </c>
-      <c r="F209" s="12" t="n"/>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Dešťová voda je u referenční realizace řešena zásakem.</t>
+        </is>
+      </c>
+      <c r="F209" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="210" ht="15.75" customHeight="1" s="13">
       <c r="C210" s="10" t="inlineStr">
@@ -3458,7 +3547,21 @@
           <t>Staví se dům celý na pozemku, nebo se jeho části vyrábějí předem?</t>
         </is>
       </c>
-      <c r="F220" s="12" t="n"/>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Dům je rámová dřevostavba; web však neuvádí přesný podíl výroby mimo staveniště.</t>
+        </is>
+      </c>
+      <c r="F220" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="221" ht="15.75" customHeight="1" s="13">
       <c r="C221" s="10" t="inlineStr">
@@ -3652,7 +3755,7 @@
           <t>Z čeho je nosná konstrukce domu?</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr">
+      <c r="E235" s="0" t="inlineStr">
         <is>
           <t>Dům je řešen jako rámová difuzně otevřená dřevostavba.</t>
         </is>
@@ -3662,7 +3765,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr">
+      <c r="H235" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -3679,7 +3782,7 @@
           <t>Je tento dům dřevostavba?</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr">
+      <c r="E236" s="0" t="inlineStr">
         <is>
           <t>Ano. Bungalov 4KK je rámová difuzně otevřená dřevostavba.</t>
         </is>
@@ -3689,7 +3792,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr">
+      <c r="H236" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -4432,7 +4535,21 @@
           <t>Je střecha připravená pro fotovoltaiku?</t>
         </is>
       </c>
-      <c r="F293" s="12" t="n"/>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Dům má integrovanou fotovoltaiku LINDAB SolarRoof.</t>
+        </is>
+      </c>
+      <c r="F293" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="294" ht="15.75" customHeight="1" s="13">
       <c r="C294" s="10" t="inlineStr">
@@ -4445,7 +4562,21 @@
           <t>Lze na střechu dodatečně instalovat fotovoltaické panely?</t>
         </is>
       </c>
-      <c r="F294" s="12" t="n"/>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Na domě je použita integrovaná fotovoltaika LINDAB SolarRoof.</t>
+        </is>
+      </c>
+      <c r="F294" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="295" ht="15.75" customHeight="1" s="13">
       <c r="C295" s="10" t="inlineStr">
@@ -4498,7 +4629,7 @@
           <t>Jaká okna jsou v domě použitá?</t>
         </is>
       </c>
-      <c r="E298" t="inlineStr">
+      <c r="E298" s="0" t="inlineStr">
         <is>
           <t>Jsou použita plastová okna s trojitým zasklením.</t>
         </is>
@@ -4508,7 +4639,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H298" t="inlineStr">
+      <c r="H298" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -4525,7 +4656,7 @@
           <t>Jsou okna s dvojsklem, nebo trojsklem?</t>
         </is>
       </c>
-      <c r="E299" t="inlineStr">
+      <c r="E299" s="0" t="inlineStr">
         <is>
           <t>Okna mají trojité zasklení.</t>
         </is>
@@ -4535,7 +4666,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H299" t="inlineStr">
+      <c r="H299" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -4552,7 +4683,7 @@
           <t>Z jakého materiálu jsou okenní rámy?</t>
         </is>
       </c>
-      <c r="E300" t="inlineStr">
+      <c r="E300" s="0" t="inlineStr">
         <is>
           <t>Okenní rámy jsou plastové.</t>
         </is>
@@ -4562,7 +4693,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H300" t="inlineStr">
+      <c r="H300" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5107,7 +5238,7 @@
           <t>Jakou požární odolnost mají stěny a další konstrukce domu?</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr">
+      <c r="E341" s="0" t="inlineStr">
         <is>
           <t>Web uvádí vysokou požární odolnost, ale konkrétní požární klasifikaci neuvádí.</t>
         </is>
@@ -5117,7 +5248,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H341" t="inlineStr">
+      <c r="H341" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5348,7 +5479,21 @@
           <t>Splňuje dům všechny požadované požární a bezpečnostní normy?</t>
         </is>
       </c>
-      <c r="F358" s="12" t="n"/>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Web uvádí vysokou požární odolnost, konkrétní normové hodnoty ale neuvádí.</t>
+        </is>
+      </c>
+      <c r="F358" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="359" ht="15.75" customHeight="1" s="13">
       <c r="A359" s="5" t="n"/>
@@ -5388,7 +5533,21 @@
           <t>Jak jsou v domě řešené rozvody elektřiny?</t>
         </is>
       </c>
-      <c r="F361" s="12" t="n"/>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Elektroinstalace referenční realizace zahrnuje 230 V, 400 V a fotovoltaiku LINDAB SolarRoof.</t>
+        </is>
+      </c>
+      <c r="F361" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="362" ht="15.75" customHeight="1" s="13">
       <c r="C362" s="10" t="inlineStr">
@@ -5401,7 +5560,21 @@
           <t>Jak jsou řešené rozvody vody?</t>
         </is>
       </c>
-      <c r="F362" s="12" t="n"/>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Dům je napojen na dálkový vodovod.</t>
+        </is>
+      </c>
+      <c r="F362" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="363" ht="15.75" customHeight="1" s="13">
       <c r="C363" s="10" t="inlineStr">
@@ -5414,7 +5587,7 @@
           <t>Jak je dům napojený na kanalizaci?</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr">
+      <c r="E363" s="0" t="inlineStr">
         <is>
           <t>U referenční realizace DŮM 002 je odpad řešen biologickou čističkou a zásakem dešťové vody.</t>
         </is>
@@ -5424,7 +5597,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H363" t="inlineStr">
+      <c r="H363" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5506,19 +5679,24 @@
           <t>Je možné doplnit chytré řízení domácnosti?</t>
         </is>
       </c>
-      <c r="E369" t="inlineStr">
+      <c r="E369" s="0" t="inlineStr">
         <is>
           <t>Ano. Referenční realizace je řízena systémem LOXONE.</t>
         </is>
       </c>
       <c r="F369" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H369" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>DSE web nedokládá, zda je dům připravený pro nabíjení elektromobilu.</t>
+        </is>
+      </c>
+      <c r="H369" s="0" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5711,21 @@
           <t>Jak je připravené internetové a datové připojení?</t>
         </is>
       </c>
-      <c r="F370" s="12" t="n"/>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Ano. Referenční realizace používá systém chytrého řízení LOXONE.</t>
+        </is>
+      </c>
+      <c r="F370" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="371" ht="15.75" customHeight="1" s="13">
       <c r="C371" s="10" t="inlineStr">
@@ -5546,7 +5738,21 @@
           <t>Jak je řešený rozvod teplé vody?</t>
         </is>
       </c>
-      <c r="F371" s="12" t="n"/>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Ohřev a akumulace tepla jsou spojeny s tepelným čerpadlem a tepelným zásobníkem; web detail rozvodu teplé vody nepopisuje.</t>
+        </is>
+      </c>
+      <c r="F371" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="372" ht="15.75" customHeight="1" s="13">
       <c r="C372" s="10" t="inlineStr">
@@ -5658,7 +5864,21 @@
           <t>Které technické instalace vyžadují pravidelné revize?</t>
         </is>
       </c>
-      <c r="F379" s="12" t="n"/>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Web neuvádí konkrétní seznam pravidelných revizí technických instalací.</t>
+        </is>
+      </c>
+      <c r="F379" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="380" ht="15.75" customHeight="1" s="13">
       <c r="A380" s="5" t="n"/>
@@ -5698,7 +5918,7 @@
           <t>Čím se tento dům vytápí?</t>
         </is>
       </c>
-      <c r="E382" t="inlineStr">
+      <c r="E382" s="0" t="inlineStr">
         <is>
           <t>Vytápění zajišťuje tepelné čerpadlo doplněné krbem s tepelným zásobníkem.</t>
         </is>
@@ -5708,7 +5928,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H382" t="inlineStr">
+      <c r="H382" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5725,7 +5945,21 @@
           <t>Jaký systém vytápění je v domě použitý?</t>
         </is>
       </c>
-      <c r="F383" s="12" t="n"/>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Vytápění zajišťuje tepelné čerpadlo a dvouplášťový krb napojený na zásobník tepla.</t>
+        </is>
+      </c>
+      <c r="F383" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="384" ht="15.75" customHeight="1" s="13">
       <c r="C384" s="10" t="inlineStr">
@@ -5751,7 +5985,7 @@
           <t>Je v domě tepelné čerpadlo?</t>
         </is>
       </c>
-      <c r="E385" t="inlineStr">
+      <c r="E385" s="0" t="inlineStr">
         <is>
           <t>Ano. Dům používá tepelné čerpadlo.</t>
         </is>
@@ -5761,7 +5995,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H385" t="inlineStr">
+      <c r="H385" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5778,7 +6012,21 @@
           <t>Jak se v domě větrá?</t>
         </is>
       </c>
-      <c r="F386" s="12" t="n"/>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Dům využívá rekuperaci tepla ze vzduchu a šedé vody.</t>
+        </is>
+      </c>
+      <c r="F386" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="387" ht="15.75" customHeight="1" s="13">
       <c r="C387" s="10" t="inlineStr">
@@ -5791,7 +6039,7 @@
           <t>Má dům rekuperaci?</t>
         </is>
       </c>
-      <c r="E387" t="inlineStr">
+      <c r="E387" s="0" t="inlineStr">
         <is>
           <t>Ano. Dům využívá rekuperaci tepla ze vzduchu a šedé vody.</t>
         </is>
@@ -5801,7 +6049,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H387" t="inlineStr">
+      <c r="H387" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5818,7 +6066,7 @@
           <t>Dá se v domě v létě chladit?</t>
         </is>
       </c>
-      <c r="E388" t="inlineStr">
+      <c r="E388" s="0" t="inlineStr">
         <is>
           <t>Ano. Tepelné čerpadlo funguje v létě také jako klimatizace.</t>
         </is>
@@ -5828,7 +6076,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H388" t="inlineStr">
+      <c r="H388" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5845,7 +6093,21 @@
           <t>Je klimatizace součástí domu?</t>
         </is>
       </c>
-      <c r="F389" s="12" t="n"/>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Tepelné čerpadlo funguje v létě také jako klimatizace.</t>
+        </is>
+      </c>
+      <c r="F389" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="390" ht="15.75" customHeight="1" s="13">
       <c r="C390" s="10" t="inlineStr">
@@ -5938,7 +6200,21 @@
           <t>Kde jsou technologie umístěné?</t>
         </is>
       </c>
-      <c r="F396" s="12" t="n"/>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Technologie zahrnují tepelné čerpadlo, rekuperaci, krb s tepelným zásobníkem, fotovoltaiku a řízení LOXONE.</t>
+        </is>
+      </c>
+      <c r="F396" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="397" ht="15.75" customHeight="1" s="13">
       <c r="A397" s="5" t="n"/>
@@ -6038,7 +6314,7 @@
           <t>Jaké podlahy jsou v domě použité?</t>
         </is>
       </c>
-      <c r="E403" t="inlineStr">
+      <c r="E403" s="0" t="inlineStr">
         <is>
           <t>V domě jsou použity trojvrstvé dřevěné podlahy.</t>
         </is>
@@ -6048,7 +6324,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H403" t="inlineStr">
+      <c r="H403" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -9345,7 +9621,7 @@
           <t>Jakou energetickou třídu dům má?</t>
         </is>
       </c>
-      <c r="E637" t="inlineStr">
+      <c r="E637" s="0" t="inlineStr">
         <is>
           <t>Web uvádí energetickou třídu A – mimořádně úsporná.</t>
         </is>
@@ -9355,7 +9631,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H637" t="inlineStr">
+      <c r="H637" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -9494,7 +9770,21 @@
           <t>Je možné spotřebu domu snížit fotovoltaikou?</t>
         </is>
       </c>
-      <c r="F646" s="12" t="n"/>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Dům má integrovanou fotovoltaiku LINDAB SolarRoof.</t>
+        </is>
+      </c>
+      <c r="F646" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="647" ht="15.75" customHeight="1" s="13">
       <c r="A647" s="5" t="n"/>
@@ -9509,7 +9799,21 @@
           <t>Je dům na instalaci fotovoltaiky připravený?</t>
         </is>
       </c>
-      <c r="F647" s="12" t="n"/>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Fotovoltaika LINDAB SolarRoof je součástí referenční realizace.</t>
+        </is>
+      </c>
+      <c r="F647" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="648" ht="15.75" customHeight="1" s="13">
       <c r="A648" s="5" t="n"/>

</xml_diff>

<commit_message>
docs(knowledge): repair DSE knowledge mappings
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
+++ b/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
@@ -1408,7 +1408,7 @@
           <t>Jaká je užitná plocha domu?</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="0" t="inlineStr">
         <is>
           <t>Užitná plocha domu je uvedena jako 129 m².</t>
         </is>
@@ -1418,7 +1418,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -1437,7 +1437,7 @@
           <t>Jaká je zastavěná plocha domu?</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="0" t="inlineStr">
         <is>
           <t>Zastavěná plocha domu je 119 m².</t>
         </is>
@@ -1447,7 +1447,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H66" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -1526,7 +1526,7 @@
           <t>Jaká je celková velikost tohoto domu?</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E71" s="0" t="inlineStr">
         <is>
           <t>Web uvádí u domu údaj 113 m², ale bez jednoznačného označení typu plochy.</t>
         </is>
@@ -1536,12 +1536,12 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
+      <c r="G71" s="0" t="inlineStr">
         <is>
           <t>Zastavěná plocha 119 m² / Užitná plocha 129 m²</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H71" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -3246,7 +3246,7 @@
           <t>Jak se dům napojuje na elektřinu, vodu a kanalizaci?</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr">
+      <c r="E200" s="0" t="inlineStr">
         <is>
           <t>Referenční realizace má dálkový vodovod, elektřinu 230/400 V a biologickou čističku odpadních vod.</t>
         </is>
@@ -3256,7 +3256,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr">
+      <c r="H200" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -3273,7 +3273,7 @@
           <t>Co když na pozemku není kanalizace?</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E201" s="0" t="inlineStr">
         <is>
           <t>Referenční realizace používá biologickou čističku odpadních vod.</t>
         </is>
@@ -3283,7 +3283,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr">
+      <c r="H201" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -3391,7 +3391,7 @@
           <t>Jak se řeší dešťová voda ze střechy?</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr">
+      <c r="E209" s="0" t="inlineStr">
         <is>
           <t>Dešťová voda je u referenční realizace řešena zásakem.</t>
         </is>
@@ -3401,7 +3401,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr">
+      <c r="H209" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -3547,7 +3547,7 @@
           <t>Staví se dům celý na pozemku, nebo se jeho části vyrábějí předem?</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr">
+      <c r="E220" s="0" t="inlineStr">
         <is>
           <t>Dům je rámová dřevostavba; web však neuvádí přesný podíl výroby mimo staveniště.</t>
         </is>
@@ -3557,7 +3557,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr">
+      <c r="H220" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -4535,7 +4535,7 @@
           <t>Je střecha připravená pro fotovoltaiku?</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr">
+      <c r="E293" s="0" t="inlineStr">
         <is>
           <t>Dům má integrovanou fotovoltaiku LINDAB SolarRoof.</t>
         </is>
@@ -4545,7 +4545,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr">
+      <c r="H293" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -4562,21 +4562,9 @@
           <t>Lze na střechu dodatečně instalovat fotovoltaické panely?</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>Na domě je použita integrovaná fotovoltaika LINDAB SolarRoof.</t>
-        </is>
-      </c>
-      <c r="F294" s="12" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H294" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="E294" s="0" t="n"/>
+      <c r="F294" s="12" t="n"/>
+      <c r="H294" s="0" t="n"/>
     </row>
     <row r="295" ht="15.75" customHeight="1" s="13">
       <c r="C295" s="10" t="inlineStr">
@@ -5479,7 +5467,7 @@
           <t>Splňuje dům všechny požadované požární a bezpečnostní normy?</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr">
+      <c r="E358" s="0" t="inlineStr">
         <is>
           <t>Web uvádí vysokou požární odolnost, konkrétní normové hodnoty ale neuvádí.</t>
         </is>
@@ -5489,7 +5477,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr">
+      <c r="H358" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5533,7 +5521,7 @@
           <t>Jak jsou v domě řešené rozvody elektřiny?</t>
         </is>
       </c>
-      <c r="E361" t="inlineStr">
+      <c r="E361" s="0" t="inlineStr">
         <is>
           <t>Elektroinstalace referenční realizace zahrnuje 230 V, 400 V a fotovoltaiku LINDAB SolarRoof.</t>
         </is>
@@ -5543,7 +5531,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H361" t="inlineStr">
+      <c r="H361" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5560,7 +5548,7 @@
           <t>Jak jsou řešené rozvody vody?</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr">
+      <c r="E362" s="0" t="inlineStr">
         <is>
           <t>Dům je napojen na dálkový vodovod.</t>
         </is>
@@ -5570,7 +5558,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H362" t="inlineStr">
+      <c r="H362" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5681,22 +5669,18 @@
       </c>
       <c r="E369" s="0" t="inlineStr">
         <is>
-          <t>Ano. Referenční realizace je řízena systémem LOXONE.</t>
+          <t>Ano. Referenční realizace používá systém chytrého řízení LOXONE.</t>
         </is>
       </c>
       <c r="F369" s="12" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G369" t="inlineStr">
-        <is>
-          <t>DSE web nedokládá, zda je dům připravený pro nabíjení elektromobilu.</t>
-        </is>
-      </c>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G369" s="0" t="n"/>
       <c r="H369" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
       </c>
     </row>
@@ -5711,9 +5695,9 @@
           <t>Jak je připravené internetové a datové připojení?</t>
         </is>
       </c>
-      <c r="E370" t="inlineStr">
-        <is>
-          <t>Ano. Referenční realizace používá systém chytrého řízení LOXONE.</t>
+      <c r="E370" s="0" t="inlineStr">
+        <is>
+          <t>Referenční realizace má internetové připojení a kabelové rozvody.</t>
         </is>
       </c>
       <c r="F370" s="12" t="inlineStr">
@@ -5721,7 +5705,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H370" t="inlineStr">
+      <c r="H370" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5738,7 +5722,7 @@
           <t>Jak je řešený rozvod teplé vody?</t>
         </is>
       </c>
-      <c r="E371" t="inlineStr">
+      <c r="E371" s="0" t="inlineStr">
         <is>
           <t>Ohřev a akumulace tepla jsou spojeny s tepelným čerpadlem a tepelným zásobníkem; web detail rozvodu teplé vody nepopisuje.</t>
         </is>
@@ -5748,7 +5732,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H371" t="inlineStr">
+      <c r="H371" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5864,7 +5848,7 @@
           <t>Které technické instalace vyžadují pravidelné revize?</t>
         </is>
       </c>
-      <c r="E379" t="inlineStr">
+      <c r="E379" s="0" t="inlineStr">
         <is>
           <t>Web neuvádí konkrétní seznam pravidelných revizí technických instalací.</t>
         </is>
@@ -5874,7 +5858,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H379" t="inlineStr">
+      <c r="H379" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -5945,7 +5929,7 @@
           <t>Jaký systém vytápění je v domě použitý?</t>
         </is>
       </c>
-      <c r="E383" t="inlineStr">
+      <c r="E383" s="0" t="inlineStr">
         <is>
           <t>Vytápění zajišťuje tepelné čerpadlo a dvouplášťový krb napojený na zásobník tepla.</t>
         </is>
@@ -5955,7 +5939,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H383" t="inlineStr">
+      <c r="H383" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -6012,7 +5996,7 @@
           <t>Jak se v domě větrá?</t>
         </is>
       </c>
-      <c r="E386" t="inlineStr">
+      <c r="E386" s="0" t="inlineStr">
         <is>
           <t>Dům využívá rekuperaci tepla ze vzduchu a šedé vody.</t>
         </is>
@@ -6022,7 +6006,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H386" t="inlineStr">
+      <c r="H386" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -6093,7 +6077,7 @@
           <t>Je klimatizace součástí domu?</t>
         </is>
       </c>
-      <c r="E389" t="inlineStr">
+      <c r="E389" s="0" t="inlineStr">
         <is>
           <t>Tepelné čerpadlo funguje v létě také jako klimatizace.</t>
         </is>
@@ -6103,7 +6087,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H389" t="inlineStr">
+      <c r="H389" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -6200,7 +6184,7 @@
           <t>Kde jsou technologie umístěné?</t>
         </is>
       </c>
-      <c r="E396" t="inlineStr">
+      <c r="E396" s="0" t="inlineStr">
         <is>
           <t>Technologie zahrnují tepelné čerpadlo, rekuperaci, krb s tepelným zásobníkem, fotovoltaiku a řízení LOXONE.</t>
         </is>
@@ -6210,7 +6194,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H396" t="inlineStr">
+      <c r="H396" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -9770,7 +9754,7 @@
           <t>Je možné spotřebu domu snížit fotovoltaikou?</t>
         </is>
       </c>
-      <c r="E646" t="inlineStr">
+      <c r="E646" s="0" t="inlineStr">
         <is>
           <t>Dům má integrovanou fotovoltaiku LINDAB SolarRoof.</t>
         </is>
@@ -9780,7 +9764,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H646" t="inlineStr">
+      <c r="H646" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -9799,7 +9783,7 @@
           <t>Je dům na instalaci fotovoltaiky připravený?</t>
         </is>
       </c>
-      <c r="E647" t="inlineStr">
+      <c r="E647" s="0" t="inlineStr">
         <is>
           <t>Fotovoltaika LINDAB SolarRoof je součástí referenční realizace.</t>
         </is>
@@ -9809,7 +9793,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H647" t="inlineStr">
+      <c r="H647" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>

</xml_diff>

<commit_message>
docs(knowledge): extend DSE reference facts
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
+++ b/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
@@ -769,7 +769,21 @@
           <t>Je dům použitelný i pro člověka se sníženou pohyblivostí?</t>
         </is>
       </c>
-      <c r="F22" s="12" t="n"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Ano. Bezbariérové řešení je možné po úpravě vstupu a terasy.</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="13">
       <c r="A23" s="8" t="n"/>
@@ -784,7 +798,21 @@
           <t>Je celý běžný život domu skutečně řešený v jednom podlaží?</t>
         </is>
       </c>
-      <c r="F23" s="12" t="n"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Dům má jedno hlavní podlaží; nad střední částí je technické podkroví.</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="13">
       <c r="A24" s="8" t="n"/>
@@ -1066,7 +1094,21 @@
           <t>Je pro tento dům výhodnější rovina, nebo může dobře fungovat i ve svahu?</t>
         </is>
       </c>
-      <c r="F42" s="12" t="n"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Referenční realizace stojí na téměř rovinaté zahradě.</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="13">
       <c r="A43" s="8" t="n"/>
@@ -1306,7 +1348,21 @@
           <t>Jak umístění domu ovlivňuje příjezd a parkování?</t>
         </is>
       </c>
-      <c r="F58" s="12" t="n"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Referenční realizace má dvě parkovací místa, z toho jedno kryté.</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="13">
       <c r="A59" s="8" t="n"/>
@@ -1366,7 +1422,21 @@
           <t>Jak okolní zástavba ovlivňuje vhodné umístění a orientaci domu?</t>
         </is>
       </c>
-      <c r="F62" s="12" t="n"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Referenční realizace je umístěna podél uliční čáry v klidné části obce.</t>
+        </is>
+      </c>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="13">
       <c r="A63" s="8" t="n"/>
@@ -3398,12 +3468,17 @@
       </c>
       <c r="F209" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>U referenční realizace je dešťová voda řešena zásakem.</t>
         </is>
       </c>
       <c r="H209" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
       </c>
     </row>
@@ -5226,21 +5301,9 @@
           <t>Jakou požární odolnost mají stěny a další konstrukce domu?</t>
         </is>
       </c>
-      <c r="E341" s="0" t="inlineStr">
-        <is>
-          <t>Web uvádí vysokou požární odolnost, ale konkrétní požární klasifikaci neuvádí.</t>
-        </is>
-      </c>
-      <c r="F341" s="12" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H341" s="0" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="E341" s="0" t="n"/>
+      <c r="F341" s="12" t="n"/>
+      <c r="H341" s="0" t="n"/>
     </row>
     <row r="342" ht="15.75" customHeight="1" s="13">
       <c r="C342" s="10" t="inlineStr">
@@ -5467,21 +5530,9 @@
           <t>Splňuje dům všechny požadované požární a bezpečnostní normy?</t>
         </is>
       </c>
-      <c r="E358" s="0" t="inlineStr">
-        <is>
-          <t>Web uvádí vysokou požární odolnost, konkrétní normové hodnoty ale neuvádí.</t>
-        </is>
-      </c>
-      <c r="F358" s="12" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H358" s="0" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="E358" s="0" t="n"/>
+      <c r="F358" s="12" t="n"/>
+      <c r="H358" s="0" t="n"/>
     </row>
     <row r="359" ht="15.75" customHeight="1" s="13">
       <c r="A359" s="5" t="n"/>
@@ -5775,7 +5826,21 @@
           <t>Jak se řeší dům, pokud na pozemku není kanalizace?</t>
         </is>
       </c>
-      <c r="F374" s="12" t="n"/>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Referenční realizace používá biologickou čističku odpadních vod.</t>
+        </is>
+      </c>
+      <c r="F374" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="375" ht="15.75" customHeight="1" s="13">
       <c r="C375" s="10" t="inlineStr">
@@ -5848,21 +5913,9 @@
           <t>Které technické instalace vyžadují pravidelné revize?</t>
         </is>
       </c>
-      <c r="E379" s="0" t="inlineStr">
-        <is>
-          <t>Web neuvádí konkrétní seznam pravidelných revizí technických instalací.</t>
-        </is>
-      </c>
-      <c r="F379" s="12" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H379" s="0" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="E379" s="0" t="n"/>
+      <c r="F379" s="12" t="n"/>
+      <c r="H379" s="0" t="n"/>
     </row>
     <row r="380" ht="15.75" customHeight="1" s="13">
       <c r="A380" s="5" t="n"/>
@@ -9070,7 +9123,21 @@
           <t>Jak velkou část pozemku dům ponechá pro zahradu?</t>
         </is>
       </c>
-      <c r="F600" s="12" t="n"/>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>U referenční realizace má pozemek 1015 m² a zahrada 815 m².</t>
+        </is>
+      </c>
+      <c r="F600" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
     </row>
     <row r="601" ht="15.75" customHeight="1" s="13">
       <c r="A601" s="5" t="n"/>
@@ -9607,7 +9674,7 @@
       </c>
       <c r="E637" s="0" t="inlineStr">
         <is>
-          <t>Web uvádí energetickou třídu A – mimořádně úsporná.</t>
+          <t>Dům je zařazen do energetické třídy A – mimořádně úsporná.</t>
         </is>
       </c>
       <c r="F637" s="12" t="inlineStr">

</xml_diff>

<commit_message>
docs(knowledge): normalize DSE rainwater fact
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
+++ b/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
@@ -769,7 +769,7 @@
           <t>Je dům použitelný i pro člověka se sníženou pohyblivostí?</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>Ano. Bezbariérové řešení je možné po úpravě vstupu a terasy.</t>
         </is>
@@ -779,7 +779,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -798,7 +798,7 @@
           <t>Je celý běžný život domu skutečně řešený v jednom podlaží?</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>Dům má jedno hlavní podlaží; nad střední částí je technické podkroví.</t>
         </is>
@@ -808,7 +808,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -1094,7 +1094,7 @@
           <t>Je pro tento dům výhodnější rovina, nebo může dobře fungovat i ve svahu?</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>Referenční realizace stojí na téměř rovinaté zahradě.</t>
         </is>
@@ -1104,7 +1104,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -1348,7 +1348,7 @@
           <t>Jak umístění domu ovlivňuje příjezd a parkování?</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="0" t="inlineStr">
         <is>
           <t>Referenční realizace má dvě parkovací místa, z toho jedno kryté.</t>
         </is>
@@ -1358,7 +1358,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H58" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -1422,7 +1422,7 @@
           <t>Jak okolní zástavba ovlivňuje vhodné umístění a orientaci domu?</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="0" t="inlineStr">
         <is>
           <t>Referenční realizace je umístěna podél uliční čáry v klidné části obce.</t>
         </is>
@@ -1432,7 +1432,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H62" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -3468,17 +3468,13 @@
       </c>
       <c r="F209" s="12" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G209" t="inlineStr">
-        <is>
-          <t>U referenční realizace je dešťová voda řešena zásakem.</t>
-        </is>
-      </c>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G209" s="0" t="n"/>
       <c r="H209" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5822,7 @@
           <t>Jak se řeší dům, pokud na pozemku není kanalizace?</t>
         </is>
       </c>
-      <c r="E374" t="inlineStr">
+      <c r="E374" s="0" t="inlineStr">
         <is>
           <t>Referenční realizace používá biologickou čističku odpadních vod.</t>
         </is>
@@ -5836,7 +5832,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H374" t="inlineStr">
+      <c r="H374" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>
@@ -9123,7 +9119,7 @@
           <t>Jak velkou část pozemku dům ponechá pro zahradu?</t>
         </is>
       </c>
-      <c r="E600" t="inlineStr">
+      <c r="E600" s="0" t="inlineStr">
         <is>
           <t>U referenční realizace má pozemek 1015 m² a zahrada 815 m².</t>
         </is>
@@ -9133,7 +9129,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H600" t="inlineStr">
+      <c r="H600" s="0" t="inlineStr">
         <is>
           <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
         </is>

</xml_diff>

<commit_message>
docs(knowledge): ingest Bungalov 4KK technical report
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
+++ b/docs/knowledge/znalostní báze – mustr 01 (1).xlsx
@@ -499,7 +499,21 @@
           <t>Pro kolik lidí je dům pohodlný pro každodenní bydlení?</t>
         </is>
       </c>
-      <c r="F4" s="12" t="n"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace počítá s trvalým bydlením pěti osob.</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 15 a 18</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="13">
       <c r="A5" s="8" t="n"/>
@@ -776,12 +790,17 @@
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace neřeší dům jako stavbu určenou pro užívání osobami se sníženou schopností pohybu nebo orientace.</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 12, 18 a 26</t>
         </is>
       </c>
     </row>
@@ -1101,12 +1120,17 @@
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Referenční pozemek je mírně svažitý a klesá směrem k jihovýchodu; při dokončovacích pracích se počítá s terénními úpravami a násypem.</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26</t>
         </is>
       </c>
     </row>
@@ -1355,12 +1379,17 @@
       </c>
       <c r="F58" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Referenční Bungalov 4KK má navržena dvě krytá odstavná stání.</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 26</t>
         </is>
       </c>
     </row>
@@ -1485,12 +1514,17 @@
       </c>
       <c r="F65" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace uvádí vytápěnou užitnou plochu 112,9 m², nevytápěnou 53,8 m² a celkovou užitnou plochu 166,7 m².</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 14–15</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1548,17 @@
       </c>
       <c r="F66" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace uvádí pro SO 2.1 Rodinný dům 4KK včetně krytého stání zastavěnou plochu 237 m².</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 2 a 14</t>
         </is>
       </c>
     </row>
@@ -3468,13 +3507,17 @@
       </c>
       <c r="F209" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="G209" s="0" t="n"/>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G209" s="0" t="inlineStr">
+        <is>
+          <t>Dešťová voda ze střechy je jímána do retenční nádrže o objemu 12 m³, filtrována a využívána pro splachování WC a závlahu; přebytek odtéká bezpečnostním přepadem do vsaku.</t>
+        </is>
+      </c>
       <c r="H209" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 15 a 30–31</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4118,21 @@
           <t>Jak je konstrukce chráněná před vlhkostí?</t>
         </is>
       </c>
-      <c r="F252" s="12" t="n"/>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Spodní stavba je chráněna natavovanými asfaltovými hydroizolačními pásy na podkladním betonu.</t>
+        </is>
+      </c>
+      <c r="F252" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="253" ht="15.75" customHeight="1" s="13">
       <c r="C253" s="10" t="inlineStr">
@@ -4178,7 +4235,21 @@
           <t>Z čeho jsou nenosné příčky?</t>
         </is>
       </c>
-      <c r="F260" s="12" t="n"/>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Svislé nenosné konstrukce jsou navrženy jako systémové SDK konstrukce nebo z EKOpanelů.</t>
+        </is>
+      </c>
+      <c r="F260" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="261" ht="15.75" customHeight="1" s="13">
       <c r="C261" s="10" t="inlineStr">
@@ -4191,7 +4262,21 @@
           <t>Jak je řešená konstrukce střechy?</t>
         </is>
       </c>
-      <c r="F261" s="12" t="n"/>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Nosnou konstrukci střechy tvoří soustava dřevěných rámů z jehličnatých KVH hranolů pevnostní třídy C24.</t>
+        </is>
+      </c>
+      <c r="F261" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="15.75" customHeight="1" s="13">
       <c r="C262" s="10" t="inlineStr">
@@ -4217,7 +4302,21 @@
           <t>Jaké materiály jsou v nosné konstrukci použité?</t>
         </is>
       </c>
-      <c r="F263" s="12" t="n"/>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Nosnou konstrukci tvoří montované dřevěné rámy; střešní prvky jsou z jehličnatých KVH hranolů pevnostní třídy C24.</t>
+        </is>
+      </c>
+      <c r="F263" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="264" ht="15.75" customHeight="1" s="13">
       <c r="C264" s="10" t="inlineStr">
@@ -4243,7 +4342,21 @@
           <t>Jak je řešená parozábrana nebo parobrzda?</t>
         </is>
       </c>
-      <c r="F265" s="12" t="n"/>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Ve skladbě šikmé střechy je navržena parozábrana.</t>
+        </is>
+      </c>
+      <c r="F265" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 19</t>
+        </is>
+      </c>
     </row>
     <row r="266" ht="15.75" customHeight="1" s="13">
       <c r="C266" s="10" t="inlineStr">
@@ -4424,7 +4537,21 @@
           <t>Jaký typ střechy dům má?</t>
         </is>
       </c>
-      <c r="F279" s="12" t="n"/>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Obytná část má šikmou sedlovou střechu se sklonem 30°.</t>
+        </is>
+      </c>
+      <c r="F279" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 17–18</t>
+        </is>
+      </c>
     </row>
     <row r="280" ht="15.75" customHeight="1" s="13">
       <c r="C280" s="10" t="inlineStr">
@@ -4437,7 +4564,21 @@
           <t>Z jakého materiálu je fasáda?</t>
         </is>
       </c>
-      <c r="F280" s="12" t="n"/>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Vnější plášť je navržen z lakovaného pozinkovaného falcovaného plechu v antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F280" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 22</t>
+        </is>
+      </c>
     </row>
     <row r="281" ht="15.75" customHeight="1" s="13">
       <c r="C281" s="10" t="inlineStr">
@@ -4567,7 +4708,21 @@
           <t>Jak je řešený odvod dešťové vody ze střechy?</t>
         </is>
       </c>
-      <c r="F290" s="12" t="n"/>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Voda ze střechy je odváděna skrytými žlaby a svody do retenční nádrže; po filtraci se využívá jako užitková voda a přebytek je zasakován.</t>
+        </is>
+      </c>
+      <c r="F290" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 30–31</t>
+        </is>
+      </c>
     </row>
     <row r="291" ht="15.75" customHeight="1" s="13">
       <c r="C291" s="10" t="inlineStr">
@@ -4580,7 +4735,21 @@
           <t>Jak jsou řešené okapy a svody?</t>
         </is>
       </c>
-      <c r="F291" s="12" t="n"/>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Střešní žlaby jsou skryté a kruhové svody jsou z lakovaného pozinkovaného plechu v šedém odstínu.</t>
+        </is>
+      </c>
+      <c r="F291" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18</t>
+        </is>
+      </c>
     </row>
     <row r="292" ht="15.75" customHeight="1" s="13">
       <c r="C292" s="10" t="inlineStr">
@@ -4769,7 +4938,21 @@
           <t>Jakou barvu mají okna?</t>
         </is>
       </c>
-      <c r="F301" s="12" t="n"/>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Plastová okna jsou navržena v tmavě šedém antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F301" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18</t>
+        </is>
+      </c>
     </row>
     <row r="302" ht="15.75" customHeight="1" s="13">
       <c r="C302" s="10" t="inlineStr">
@@ -4782,7 +4965,21 @@
           <t>Jaké jsou tepelněizolační vlastnosti oken?</t>
         </is>
       </c>
-      <c r="F302" s="12" t="n"/>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Okna mají izolační trojsklo a projektová dokumentace uvádí Uw,max = 0,5 W/m²K.</t>
+        </is>
+      </c>
+      <c r="F302" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="303" ht="15.75" customHeight="1" s="13">
       <c r="C303" s="10" t="inlineStr">
@@ -4912,7 +5109,21 @@
           <t>Jaké jsou vstupní dveře do domu?</t>
         </is>
       </c>
-      <c r="F312" s="12" t="n"/>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Vstupní dveře jsou plastové v tmavě šedém antracitovém odstínu; dokumentace uvádí Ud,max = 0,6 W/m²K.</t>
+        </is>
+      </c>
+      <c r="F312" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 22</t>
+        </is>
+      </c>
     </row>
     <row r="313" ht="15.75" customHeight="1" s="13">
       <c r="C313" s="10" t="inlineStr">
@@ -5058,7 +5269,21 @@
           <t>Jaká izolace je použitá v obvodových stěnách?</t>
         </is>
       </c>
-      <c r="F323" s="12" t="n"/>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Obvodové stěny jsou zatepleny foukanou celulózovou izolací Climatizer.</t>
+        </is>
+      </c>
+      <c r="F323" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="324" ht="15.75" customHeight="1" s="13">
       <c r="C324" s="10" t="inlineStr">
@@ -5071,7 +5296,21 @@
           <t>Jaká izolace je použitá ve střeše?</t>
         </is>
       </c>
-      <c r="F324" s="12" t="n"/>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Střešní konstrukce je zateplena foukanou celulózovou izolací Climatizer.</t>
+        </is>
+      </c>
+      <c r="F324" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="325" ht="15.75" customHeight="1" s="13">
       <c r="C325" s="10" t="inlineStr">
@@ -5084,7 +5323,21 @@
           <t>Jak je zateplená podlaha?</t>
         </is>
       </c>
-      <c r="F325" s="12" t="n"/>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Podlaha na terénu je podle projektové dokumentace zateplena foukanou celulózovou izolací Climatizer.</t>
+        </is>
+      </c>
+      <c r="F325" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="326" ht="15.75" customHeight="1" s="13">
       <c r="C326" s="10" t="inlineStr">
@@ -5629,12 +5882,17 @@
       </c>
       <c r="F363" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Referenční realizace není napojena na veřejnou splaškovou kanalizaci; odpadní vody jsou vedeny do certifikované domovní ČOV Aquatec AT8 a přečištěná voda následně do zasakovacího systému.</t>
         </is>
       </c>
       <c r="H363" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 30; A Průvodní zpráva, str. 4</t>
         </is>
       </c>
     </row>
@@ -6005,7 +6263,21 @@
           <t>Má dům podlahové vytápění?</t>
         </is>
       </c>
-      <c r="F384" s="12" t="n"/>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Ne. Projektová dokumentace výslovně uvádí, že podlahové vytápění není součástí kontaktní konstrukce.</t>
+        </is>
+      </c>
+      <c r="F384" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 24</t>
+        </is>
+      </c>
     </row>
     <row r="385" ht="15.75" customHeight="1" s="13">
       <c r="C385" s="10" t="inlineStr">
@@ -6192,7 +6464,21 @@
           <t>Musím při rekuperaci otevírat okna?</t>
         </is>
       </c>
-      <c r="F393" s="12" t="n"/>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Ne. Běžné větrání zajišťuje nucená rekuperace; okna a dveře lze otevřít pro příležitostné přirozené větrání.</t>
+        </is>
+      </c>
+      <c r="F393" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 24</t>
+        </is>
+      </c>
     </row>
     <row r="394" ht="15.75" customHeight="1" s="13">
       <c r="C394" s="10" t="inlineStr">
@@ -6205,7 +6491,21 @@
           <t>Je možné větrat normálně okny i při použití rekuperace?</t>
         </is>
       </c>
-      <c r="F394" s="12" t="n"/>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Ano. Projektová dokumentace počítá s nuceným větráním rekuperací i s možností příležitostného větrání otevřenými okny nebo dveřmi.</t>
+        </is>
+      </c>
+      <c r="F394" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 24</t>
+        </is>
+      </c>
     </row>
     <row r="395" ht="15.75" customHeight="1" s="13">
       <c r="C395" s="10" t="inlineStr">
@@ -6354,12 +6654,17 @@
       </c>
       <c r="F403" s="12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace navrhuje nášlapné vrstvy z vinylových lamel a keramické dlažby.</t>
         </is>
       </c>
       <c r="H403" s="0" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 18 a 22</t>
         </is>
       </c>
     </row>
@@ -6517,7 +6822,21 @@
           <t>Jsou mezi místnostmi prahy?</t>
         </is>
       </c>
-      <c r="F415" s="12" t="n"/>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace počítá s dveřními prahy z dubového dřeva.</t>
+        </is>
+      </c>
+      <c r="F415" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
     </row>
     <row r="416" ht="15.75" customHeight="1" s="13">
       <c r="A416" s="5" t="n"/>
@@ -9033,7 +9352,21 @@
           <t>Je terasa součástí základního řešení domu?</t>
         </is>
       </c>
-      <c r="F594" s="12" t="n"/>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Referenční projekt obsahuje krytou terasu o rozměrech 3 × 10 m.</t>
+        </is>
+      </c>
+      <c r="F594" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>A Průvodní zpráva, str. 3; B Souhrnná technická zpráva 11/2023, str. 17–18</t>
+        </is>
+      </c>
     </row>
     <row r="595" ht="15.75" customHeight="1" s="13">
       <c r="C595" s="10" t="inlineStr">
@@ -9362,7 +9695,21 @@
           <t>Jak dobře dům tlumí hluk zvenčí?</t>
         </is>
       </c>
-      <c r="F616" s="12" t="n"/>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Obvodový plášť je navržen tak, aby splňoval požadavky na běžnou akustickou ochranu budovy podle ČSN 73 0532.</t>
+        </is>
+      </c>
+      <c r="F616" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 25</t>
+        </is>
+      </c>
     </row>
     <row r="617" ht="15.75" customHeight="1" s="13">
       <c r="A617" s="5" t="n"/>

</xml_diff>